<commit_message>
fixing bug where switching presence annotations did not update details page.
</commit_message>
<xml_diff>
--- a/data/source/codebook.xlsx
+++ b/data/source/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/human_annotation_tool/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A04108B-528F-5340-BCDE-1C8A174E4A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6D5E9E-9369-4C46-A550-8E70F8F94229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core_Schema_SIMPLIFIED" sheetId="1" r:id="rId1"/>
@@ -86,9 +86,6 @@
     <t>KS_evidence_present</t>
   </si>
   <si>
-    <t>Whether the contributor invokes an identifiable evidence item in support of the claim.</t>
-  </si>
-  <si>
     <t>Raw text: “Oxford English Dictionary ‘non-combatant’ … A person who is not a combatant, as a civilian during a war…”
 Explanation: The contributor invokes a specifically identifiable external source as evidence.</t>
   </si>
@@ -727,6 +724,9 @@
   </si>
   <si>
     <t>Whether the contributor asks others to assess, revise, or accept, their work.</t>
+  </si>
+  <si>
+    <t>Whether the contributor invokes (or references) an identifiable evidence item.</t>
   </si>
 </sst>
 </file>
@@ -1023,10 +1023,10 @@
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>16</v>
@@ -1046,13 +1046,13 @@
         <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>17</v>
@@ -1063,22 +1063,22 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="140.75" customHeight="1">
@@ -1086,22 +1086,22 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="F6" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="258" customHeight="1">
@@ -1109,22 +1109,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="117.25" customHeight="1">
@@ -1132,42 +1132,42 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="117.25" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>17</v>
@@ -1175,22 +1175,22 @@
     </row>
     <row r="10" spans="1:7" ht="117.25" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>17</v>
@@ -1198,22 +1198,22 @@
     </row>
     <row r="11" spans="1:7" ht="117.25" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>
@@ -1221,91 +1221,91 @@
     </row>
     <row r="12" spans="1:7" ht="117.25" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>205</v>
-      </c>
       <c r="F12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="117.25" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>209</v>
-      </c>
       <c r="E13" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="164.25" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="D14" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>211</v>
-      </c>
       <c r="G14" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="117.25" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>13</v>
@@ -1313,91 +1313,91 @@
     </row>
     <row r="16" spans="1:7" ht="117.25" customHeight="1">
       <c r="A16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="117.25" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="117.25" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="G18" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="117.25" customHeight="1">
       <c r="A19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>13</v>
@@ -1455,10 +1455,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>12</v>
@@ -1478,10 +1478,10 @@
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>16</v>
@@ -1501,13 +1501,13 @@
         <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>17</v>
@@ -1518,22 +1518,22 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="123.25" customHeight="1">
@@ -1541,22 +1541,22 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="193.5" customHeight="1">
@@ -1564,22 +1564,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="105.5" customHeight="1">
@@ -1587,42 +1587,42 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="88" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>89</v>
-      </c>
       <c r="F9" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>17</v>
@@ -1630,22 +1630,22 @@
     </row>
     <row r="10" spans="1:7" ht="88" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>17</v>
@@ -1653,22 +1653,22 @@
     </row>
     <row r="11" spans="1:7" ht="88" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>
@@ -1676,91 +1676,91 @@
     </row>
     <row r="12" spans="1:7" ht="88" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="88" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="G13" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="123.25" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="88" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>13</v>
@@ -1768,91 +1768,91 @@
     </row>
     <row r="16" spans="1:7" ht="88" customHeight="1">
       <c r="A16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="F16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="88" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="105.5" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="88" customHeight="1">
       <c r="A19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="D19" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>13</v>
@@ -1877,16 +1877,16 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
@@ -1897,142 +1897,142 @@
     </row>
     <row r="2" spans="1:6" ht="70.25" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="47" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="70.25" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>114</v>
-      </c>
       <c r="F4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="70.25" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="70.25" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="F6" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="70.25" customHeight="1">
       <c r="A7" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="F7" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="70.25" customHeight="1">
       <c r="A8" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2054,7 +2054,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -2071,138 +2071,138 @@
     </row>
     <row r="2" spans="1:5" ht="70.25" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="70.25" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="47" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>147</v>
-      </c>
       <c r="E4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="70.25" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>151</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="93.75" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="47" customHeight="1">
       <c r="A7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="70.25" customHeight="1">
       <c r="A8" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="117.25" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>167</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding codebook, gold set, app state, and completed annotations.
</commit_message>
<xml_diff>
--- a/data/source/codebook.xlsx
+++ b/data/source/codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/human_annotation_tool/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B20BEF0-CA04-F547-B786-470D95FEEB0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824EB44B-946C-3540-B6DA-79FFCFB76740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,9 +55,6 @@
     <t>binary {0,1}</t>
   </si>
   <si>
-    <t>Whether the utterance stakes dispute-relevant knowledge by asserting, challenging, qualifying, or limiting a position about the article or dispute.</t>
-  </si>
-  <si>
     <t>Code 1 when the utterance makes an article- or dispute-related knowledge claim, objection, interpretation, evaluation, or constraint public. A question counts when it asserts, presupposes, or challenges a proposition. Code 0 for headings, greetings, pure coordination, governance-only talk, claims unrelated to the article or dispute, and personal remarks with no substantive article-related position. If 0, all KS dimensions are null. If 1, code every KS dimension independently; dimensions may co-occur. KS and KI may also co-occur.</t>
   </si>
   <si>
@@ -73,9 +70,6 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
   </si>
   <si>
-    <t>Does the utterance stake dispute-relevant knowledge by asserting, challenging, qualifying, or limiting an article- or dispute-related position?</t>
-  </si>
-  <si>
     <t>KS_explicit_reasoning</t>
   </si>
   <si>
@@ -100,13 +94,7 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
   </si>
   <si>
-    <t>Does the utterance explicate an inferential link between a premise or evidence and a claim or conclusion?</t>
-  </si>
-  <si>
     <t>KS_grounding</t>
-  </si>
-  <si>
-    <t>Whether the utterance invokes identifiable evidence or a supporting basis for a stake.</t>
   </si>
   <si>
     <t>Only code if KS_present=1. Code 1 for a named, quoted, or linked source; article text or feature; edit or page history; Wikipedia policy or rule; documented consensus; or another article used as support. The evidence may be weak or contested. Code 0 for an unsupported assertion or general belief with no identifiable basis. Do not require an explanation of how the evidence supports the claim; that is KS_explicit_reasoning.</t>
@@ -124,9 +112,6 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
   </si>
   <si>
-    <t>Does the utterance invoke/reference identifiable evidence or another basis of support?</t>
-  </si>
-  <si>
     <t>KS_new_evidence</t>
   </si>
   <si>
@@ -139,10 +124,13 @@
     <t>Only code if KS_grounding=1. Code 1 if at least one supporting basis appears for the first time in the dispute; otherwise code 0. Additional quotations, facts, or elaboration from already-shared evidence do not count as new.</t>
   </si>
   <si>
-    <t>Does the utterance introduce any evidence that has not previously appeared in the dispute?</t>
-  </si>
-  <si>
     <t>KS_restaking</t>
+  </si>
+  <si>
+    <t>Whether the utterance repeats a claim, objection, criterion, or position already made earlier in the dispute without adding new information.</t>
+  </si>
+  <si>
+    <t>Only code if KS_present=1. Code 1 when an earlier stake is repeated by the same or another contributor with no meaningful new information. Minor rewording counts as repetition. Code 0 if the utterance adds new evidence, reasoning, qualification, distinction, or other information, or if it is the first occurrence of the stake.</t>
   </si>
   <si>
     <t>Verbatim excerpt: “We have many different reliable sources each stating different dates. Do you see the issue?”
@@ -155,9 +143,6 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz
 WikiDisputes archive; conv_id=253990014.204845.204845; utterance_index=21; repeats utterance_index=20
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
-  </si>
-  <si>
-    <t>Does the utterance restate a claim, objection, criterion, or position already made earlier in the dispute, without adding new information?</t>
   </si>
   <si>
     <t>KS_bounding</t>
@@ -189,12 +174,6 @@
   </si>
   <si>
     <t>KI_present</t>
-  </si>
-  <si>
-    <t>Whether the utterance translates dispute-relevant knowledge into an identifiable treatment of the shared article, by discussing, constructing, adapting, adopting, or enacting how contested material should be represented.</t>
-  </si>
-  <si>
-    <t>Code 1 only when BOTH conditions are met: (1) the utterance identifies an "article treatment" (i.e., what should be written, sourced, included, excluded, retained, relocated, structured, labeled, or displayed); AND (2) that treatment is shaped by a dispute-relevant claim, evidence item, distinction, objection, or constraint visible in the utterance or prior dialogue. The treatment may be implied, proposed, adapted, adopted, or enacted; it need not succeed or resolve the dispute. Code 0 for claims, evidence, reasoning, agreement, concession, or KS_bounding alone; requests for facts; generic process/governance steps; voting or reporting consensus alone; a vague 'this is wrong/does not belong'; or a bare revert/restoration of an already-contested version with no adaptation. A simple removal/addition counts only when it is an identifiable treatment flowing from the content problem under discussion. KS and KI may co-occur.</t>
   </si>
   <si>
     <t>Verbatim excerpt: “I've moved the element of critical evaluation into the Critical reaction section per your observation.”
@@ -221,9 +200,6 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
   </si>
   <si>
-    <t>Does the utterance translate dispute-relevant knowledge into an identifiable treatment of the shared article?</t>
-  </si>
-  <si>
     <t>Controls</t>
   </si>
   <si>
@@ -244,9 +220,6 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
   </si>
   <si>
-    <t>Does the utterance redirect discussion away from the current focal article problem to material with no plausible bearing on understanding or resolving it?</t>
-  </si>
-  <si>
     <t>C_interpersonal_attack_or_disrespect</t>
   </si>
   <si>
@@ -264,9 +237,6 @@
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
   </si>
   <si>
-    <t>Does the utterance direct insult, ridicule, contempt, disrespect, bad-faith or motive attribution, or personal devaluation at a contributor or contributor group?</t>
-  </si>
-  <si>
     <t>C_formal_governance_action</t>
   </si>
   <si>
@@ -282,9 +252,6 @@
   <si>
     <t>WikiDisputes archive; conv_id=666161089.106.106; utterance_index=4
 https://github.com/christinedekock11/wikidisputes/blob/b6f5906179724969a883ebf3012064765edf133e/data.tar.gz</t>
-  </si>
-  <si>
-    <t>Does the utterance propose, threaten, request, initiate, announce, or report moving the dispute into a recognized governance procedure or seeking authoritative intervention?</t>
   </si>
   <si>
     <t>Dispute Context</t>
@@ -309,9 +276,6 @@
 Do not infer the object from the resolution.</t>
   </si>
   <si>
-    <t>What is the main editorial question participants directly disagree about across the dispute?</t>
-  </si>
-  <si>
     <t>Dispute Outcome</t>
   </si>
   <si>
@@ -332,16 +296,52 @@
 5 = Clearly resolved: the focal disagreement is clearly treated as settled by the opposing sides and is not reopened.</t>
   </si>
   <si>
-    <t>By the end of the discussion, to what extent do the opposing sides treat the focal disagreement as settled?</t>
-  </si>
-  <si>
-    <t>Whether the utterance repeats a claim, objection, criterion, or position already made earlier in the dispute without adding new information.</t>
-  </si>
-  <si>
-    <t>Only code if KS_present=1. Code 1 when an earlier stake is repeated by the same or another contributor with no meaningful new information. Minor rewording counts as repetition. Code 0 if the utterance adds new evidence, reasoning, qualification, distinction, or other information, or if it is the first occurrence of the stake.</t>
-  </si>
-  <si>
-    <t>Does the utterance repeat a claim, objection, criterion, or position already made earlier in the dispute without adding new information?</t>
+    <t>Does it explain why a reason or evidence supports a claim?</t>
+  </si>
+  <si>
+    <t>Does it repeat an earlier position without new information?</t>
+  </si>
+  <si>
+    <t>Does it shift away from the focal article problem?</t>
+  </si>
+  <si>
+    <t>Does it attack or disrespect another contributor?</t>
+  </si>
+  <si>
+    <t>Does it invoke a formal dispute-resolution or enforcement process?</t>
+  </si>
+  <si>
+    <t>What is the dispute mainly about?</t>
+  </si>
+  <si>
+    <t>How settled is the focal disagreement by the end?</t>
+  </si>
+  <si>
+    <t>Is the evidence/support new to the dispute?</t>
+  </si>
+  <si>
+    <t>Code 1 only when BOTH conditions are met: (1) the utterance discusses an "article treatment" (i.e., what should/could be written, sourced, included, excluded, retained, relocated, structured, labeled, or displayed); AND (2) that treatment appears to be shaped by a dispute-relevant claim, evidence item, distinction, objection, or constraint visible in the utterance or prior dialogue. The treatment may be implied, proposed, adapted, adopted, or enacted; it need not succeed or resolve the dispute. Code 0 for claims, evidence, reasoning, agreement, concession, or KS_bounding alone; requests for facts; generic process/governance steps; voting or reporting consensus alone; a vague 'this is wrong/does not belong'; or a bare revert/restoration of an already-contested version with no adaptation. A simple removal/addition counts only when it is an identifiable treatment flowing from the content problem under discussion. KS and KI may co-occur.</t>
+  </si>
+  <si>
+    <t>Does it turn knowledge shared in the dispute into an article treatment?</t>
+  </si>
+  <si>
+    <t>Whether the utterance invokes identifiable evidence or a supporting basis for a staked claim</t>
+  </si>
+  <si>
+    <t>Whether the utterance stakes dispute-relevant knowledge by asserting, challenging, qualifying, or limiting a claim/position about the article or dispute.</t>
+  </si>
+  <si>
+    <t>Does the utterance assert, challenge, support, qualify, or limit a dispute-relevant knowledge claim?</t>
+  </si>
+  <si>
+    <t>Whether the utterance translates previosuly shared dispute-relevant knowledge into an identifiable treatment of the shared article, by suggesting, announcing (enactment of), coordianting, constructing, or accepting how contested material should be represented.</t>
+  </si>
+  <si>
+    <t>Does it signal conditions under which the speaker might accept a position, or revise their own?</t>
+  </si>
+  <si>
+    <t>Does it cite evidence for support?</t>
   </si>
 </sst>
 </file>
@@ -415,7 +415,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -498,20 +498,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -530,31 +516,16 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -569,7 +540,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -584,7 +555,22 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -837,304 +823,304 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="115" customHeight="1">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:8" ht="165">
+      <c r="A2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="210">
+      <c r="A3" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="130" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="D3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="180">
+      <c r="A4" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="B4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="C4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="135" customHeight="1">
-      <c r="A4" s="19" t="s">
+      <c r="G4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="60">
+      <c r="A5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="70" customHeight="1">
-      <c r="A5" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="195">
+      <c r="A6" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="342">
+      <c r="A7" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="95" customHeight="1">
-      <c r="A6" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="14" t="s">
+      <c r="C7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="E7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="409.6">
+      <c r="A8" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="220" customHeight="1">
-      <c r="A7" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="E8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H8" s="20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="105">
+      <c r="A9" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="165" customHeight="1">
-      <c r="A8" s="20" t="s">
+      <c r="B9" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="C9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="E9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="75">
+      <c r="A10" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="95" customHeight="1">
-      <c r="A9" s="21" t="s">
+      <c r="E10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="F10" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="G10" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="105">
+      <c r="A11" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="8" t="s">
+      <c r="D11" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="F11" s="6" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="110" customHeight="1">
-      <c r="A10" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="16" t="s">
+      <c r="G11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="H11" s="21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="210">
+      <c r="A12" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="B12" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="E12" s="7" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="105" customHeight="1">
-      <c r="A11" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="16" t="s">
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="22" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="300">
+      <c r="A13" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="B13" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="C13" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="D13" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="E13" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="H11" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="120" customHeight="1">
-      <c r="A12" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="11" t="s">
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="23" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="175" customHeight="1">
-      <c r="A13" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="13" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Superficial modifications to codebook text.
</commit_message>
<xml_diff>
--- a/data/source/codebook.xlsx
+++ b/data/source/codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/human_annotation_tool/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4913BD69-B921-CA40-B04D-009B1EE7DBD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81891F7F-001A-2E4A-A035-DCB784500088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -328,9 +328,6 @@
 Exclusion check: this conv_id is absent from the final WikiTactics dataset and the current gold files.</t>
   </si>
   <si>
-    <t>Does the utterance coordinate a concrete change to the Wikipedia page?</t>
-  </si>
-  <si>
     <t>KI_compromise</t>
   </si>
   <si>
@@ -352,6 +349,9 @@
   </si>
   <si>
     <t>Whether the utterance offers a compromise or accommodation intended to bridge opposed positions or restore workable cooperation. An clear attempt to find a midway between the speaker's point and the opposer's.</t>
+  </si>
+  <si>
+    <t>Does the utterance attempt to coordinate an update to the Wikipedia page?</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1008,7 @@
         <v>82</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="150" customHeight="1">
@@ -1016,25 +1016,25 @@
         <v>77</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="H9" s="21" t="s">
         <v>87</v>
-      </c>
-      <c r="H9" s="21" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="105">

</xml_diff>